<commit_message>
fixed issue with dataprovider methods
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m766693\workspace\AutomationFramework2026\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m766693\workspace\AutomationSeleniumJava\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A1EBA13-6C5C-4AA2-ACA2-AE08CD3DD5BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9D6D3B7-E42C-4343-92DA-2039D2EEAD9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="162913" refMode="R1C1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,15 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="10">
   <si>
     <t>username</t>
   </si>
   <si>
     <t>password</t>
-  </si>
-  <si>
-    <t>age</t>
   </si>
   <si>
     <t>standard_user</t>
@@ -406,18 +403,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.7265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="3.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -425,64 +421,49 @@
       <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="C2" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1">
-        <v>10</v>
+      <c r="C3" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="1" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="1">
-        <v>20</v>
+      <c r="C4" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="1">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="1">
-        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated browser to chrome
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m766693\workspace\AutomationSeleniumJava\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9D6D3B7-E42C-4343-92DA-2039D2EEAD9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5138FFA9-5DDB-4D19-97B6-168DE1D44112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="9">
   <si>
     <t>username</t>
   </si>
@@ -52,9 +52,6 @@
   </si>
   <si>
     <t>chrome</t>
-  </si>
-  <si>
-    <t>edge</t>
   </si>
 </sst>
 </file>
@@ -435,7 +432,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>3</v>
@@ -457,7 +454,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>5</v>

</xml_diff>

<commit_message>
added options to edgedriver to fix launch issue from jenkins
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m766693\workspace\AutomationSeleniumJava\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5138FFA9-5DDB-4D19-97B6-168DE1D44112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E3CB5BF-4B03-457E-A17C-8925B879B349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="10">
   <si>
     <t>username</t>
   </si>
@@ -52,6 +52,9 @@
   </si>
   <si>
     <t>chrome</t>
+  </si>
+  <si>
+    <t>edge</t>
   </si>
 </sst>
 </file>
@@ -432,7 +435,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>3</v>
@@ -454,7 +457,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>5</v>

</xml_diff>

<commit_message>
renamed Extent report name to static
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m766693\workspace\AutomationSeleniumJava\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E3CB5BF-4B03-457E-A17C-8925B879B349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDAEFEE2-9219-43D2-8BCD-34617F00E873}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="9">
   <si>
     <t>username</t>
   </si>
@@ -52,9 +52,6 @@
   </si>
   <si>
     <t>chrome</t>
-  </si>
-  <si>
-    <t>edge</t>
   </si>
 </sst>
 </file>
@@ -435,7 +432,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>3</v>
@@ -457,7 +454,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>5</v>

</xml_diff>